<commit_message>
Employee Page Test added , Adding and Deleting an Employee
</commit_message>
<xml_diff>
--- a/src/main/resources/TestData/TestData.xlsx
+++ b/src/main/resources/TestData/TestData.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Purvesh\Automation_Workspace\OrangeHRMTestNG\src\main\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{025556BC-9B0C-423A-961F-9F0A086220DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875B4C7C-EC56-4510-95D2-00B6BF645F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
     <sheet name="InValidLogin" sheetId="2" r:id="rId2"/>
     <sheet name="Employee" sheetId="3" r:id="rId3"/>
+    <sheet name="LoginAndEmployeeData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
   <si>
     <t>username</t>
   </si>
@@ -47,12 +48,6 @@
     <t>test123</t>
   </si>
   <si>
-    <t>prod</t>
-  </si>
-  <si>
-    <t>prod123</t>
-  </si>
-  <si>
     <t>Name</t>
   </si>
   <si>
@@ -93,14 +88,46 @@
   </si>
   <si>
     <t>qa123</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>MiddleName</t>
+  </si>
+  <si>
+    <t>EmployeeId</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>TName</t>
+  </si>
+  <si>
+    <t>PLastName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -149,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -158,6 +185,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -439,7 +472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
@@ -458,22 +491,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -481,7 +498,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04538036-8B4F-41A7-AB10-C35EFCF68929}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
@@ -502,18 +519,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -532,31 +541,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B4" s="4">
         <v>11223344</v>
@@ -564,10 +573,10 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.45">
@@ -575,7 +584,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.45">
@@ -583,15 +592,73 @@
         <v>1</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58058E19-D76A-437C-9CAB-45B9E5465B39}">
+  <dimension ref="A1:F2"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="16.265625" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="17.59765625" customWidth="1"/>
+    <col min="4" max="4" width="16.53125" customWidth="1"/>
+    <col min="5" max="5" width="15.3984375" customWidth="1"/>
+    <col min="6" max="6" width="16.3984375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A1" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="5">
+        <v>1122555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>